<commit_message>
chore: update analysis artifacts and add gitignore entry for stale draft
</commit_message>
<xml_diff>
--- a/Analysis/PositionBias/position_bias_summary_all_models.xlsx
+++ b/Analysis/PositionBias/position_bias_summary_all_models.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1389,902 +1389,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Qwen3.5 9B</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>195</v>
-      </c>
-      <c r="G18" t="n">
-        <v>5</v>
-      </c>
-      <c r="H18" t="n">
-        <v>56.8</v>
-      </c>
-      <c r="I18" t="n">
-        <v>27.2</v>
-      </c>
-      <c r="J18" t="n">
-        <v>-29.6</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0.0011</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0.0106</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0.3867</v>
-      </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Qwen3.5 9B</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>HVAC</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>70</v>
-      </c>
-      <c r="G19" t="n">
-        <v>5</v>
-      </c>
-      <c r="H19" t="n">
-        <v>20.2</v>
-      </c>
-      <c r="I19" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="J19" t="n">
-        <v>-9.800000000000001</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0.1221</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0.3616</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0.3686</v>
-      </c>
-      <c r="N19" t="n">
-        <v>0.2442</v>
-      </c>
-      <c r="O19" t="n">
-        <v>0.7232</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Qwen3.5 9B</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Appliance</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>65</v>
-      </c>
-      <c r="G20" t="n">
-        <v>5</v>
-      </c>
-      <c r="H20" t="n">
-        <v>16.2</v>
-      </c>
-      <c r="I20" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="J20" t="n">
-        <v>-5.8</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0.3449</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0.7010999999999999</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0.4246</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0.3449</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0.7232</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Qwen3.5 9B</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Shower</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>60</v>
-      </c>
-      <c r="G21" t="n">
-        <v>5</v>
-      </c>
-      <c r="H21" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="I21" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="J21" t="n">
-        <v>-14</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0.1078</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0.3667</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0.0075</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0.3234</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>gptoss</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>GPT-OSS 20B</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>195</v>
-      </c>
-      <c r="G22" t="n">
-        <v>5</v>
-      </c>
-      <c r="H22" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="I22" t="n">
-        <v>24</v>
-      </c>
-      <c r="J22" t="n">
-        <v>-30.6</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0.0023</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0.0043</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0.4605</v>
-      </c>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>gptoss</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>GPT-OSS 20B</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>HVAC</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>70</v>
-      </c>
-      <c r="G23" t="n">
-        <v>5</v>
-      </c>
-      <c r="H23" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="I23" t="n">
-        <v>10</v>
-      </c>
-      <c r="J23" t="n">
-        <v>-12.8</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0.041</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0.1496</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0.123</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0.4488</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>gptoss</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>GPT-OSS 20B</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Appliance</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>65</v>
-      </c>
-      <c r="G24" t="n">
-        <v>5</v>
-      </c>
-      <c r="H24" t="n">
-        <v>12.8</v>
-      </c>
-      <c r="I24" t="n">
-        <v>6</v>
-      </c>
-      <c r="J24" t="n">
-        <v>-6.8</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0.1671</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0.4545</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0.5138</v>
-      </c>
-      <c r="N24" t="n">
-        <v>0.1671</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0.459</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>gptoss</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>GPT-OSS 20B</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Shower</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>60</v>
-      </c>
-      <c r="G25" t="n">
-        <v>5</v>
-      </c>
-      <c r="H25" t="n">
-        <v>19</v>
-      </c>
-      <c r="I25" t="n">
-        <v>8</v>
-      </c>
-      <c r="J25" t="n">
-        <v>-11</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0.0755</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0.2295</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0.151</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0.459</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>deepseek</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>DeepSeek V4 Flash</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>195</v>
-      </c>
-      <c r="G26" t="n">
-        <v>5</v>
-      </c>
-      <c r="H26" t="n">
-        <v>56.2</v>
-      </c>
-      <c r="I26" t="n">
-        <v>39</v>
-      </c>
-      <c r="J26" t="n">
-        <v>-17.2</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0.079</v>
-      </c>
-      <c r="L26" t="n">
-        <v>0.3776</v>
-      </c>
-      <c r="M26" t="n">
-        <v>0.4143</v>
-      </c>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>deepseek</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>DeepSeek V4 Flash</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>HVAC</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>70</v>
-      </c>
-      <c r="G27" t="n">
-        <v>5</v>
-      </c>
-      <c r="H27" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="I27" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="J27" t="n">
-        <v>3</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0.7201</v>
-      </c>
-      <c r="L27" t="n">
-        <v>1</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0.3743</v>
-      </c>
-      <c r="N27" t="n">
-        <v>1</v>
-      </c>
-      <c r="O27" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>deepseek</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>DeepSeek V4 Flash</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Appliance</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>65</v>
-      </c>
-      <c r="G28" t="n">
-        <v>5</v>
-      </c>
-      <c r="H28" t="n">
-        <v>30.8</v>
-      </c>
-      <c r="I28" t="n">
-        <v>10.2</v>
-      </c>
-      <c r="J28" t="n">
-        <v>-20.6</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0.0051</v>
-      </c>
-      <c r="L28" t="n">
-        <v>0.0195</v>
-      </c>
-      <c r="M28" t="n">
-        <v>0.3292</v>
-      </c>
-      <c r="N28" t="n">
-        <v>0.0153</v>
-      </c>
-      <c r="O28" t="n">
-        <v>0.0585</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>deepseek</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>DeepSeek V4 Flash</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Shower</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>60</v>
-      </c>
-      <c r="G29" t="n">
-        <v>5</v>
-      </c>
-      <c r="H29" t="n">
-        <v>11.6</v>
-      </c>
-      <c r="I29" t="n">
-        <v>12</v>
-      </c>
-      <c r="J29" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="K29" t="n">
-        <v>0.8238</v>
-      </c>
-      <c r="L29" t="n">
-        <v>1</v>
-      </c>
-      <c r="M29" t="n">
-        <v>0.5533</v>
-      </c>
-      <c r="N29" t="n">
-        <v>1</v>
-      </c>
-      <c r="O29" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>gemini</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Gemini 3.5 Flash</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>193</v>
-      </c>
-      <c r="G30" t="n">
-        <v>5</v>
-      </c>
-      <c r="H30" t="n">
-        <v>37.6</v>
-      </c>
-      <c r="I30" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="J30" t="n">
-        <v>-25.8</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0.0003</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0.0016</v>
-      </c>
-      <c r="M30" t="n">
-        <v>0.6919999999999999</v>
-      </c>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>gemini</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Gemini 3.5 Flash</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>HVAC</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>69</v>
-      </c>
-      <c r="G31" t="n">
-        <v>5</v>
-      </c>
-      <c r="H31" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="I31" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="J31" t="n">
-        <v>-4.6</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0.5078</v>
-      </c>
-      <c r="L31" t="n">
-        <v>0.5488</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0.7637</v>
-      </c>
-      <c r="N31" t="n">
-        <v>1</v>
-      </c>
-      <c r="O31" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>gemini</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Gemini 3.5 Flash</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Appliance</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>65</v>
-      </c>
-      <c r="G32" t="n">
-        <v>5</v>
-      </c>
-      <c r="H32" t="n">
-        <v>24.4</v>
-      </c>
-      <c r="I32" t="n">
-        <v>3</v>
-      </c>
-      <c r="J32" t="n">
-        <v>-21.4</v>
-      </c>
-      <c r="K32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="M32" t="n">
-        <v>0.5091</v>
-      </c>
-      <c r="N32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O32" t="n">
-        <v>0.0003</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>gemini</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Gemini 3.5 Flash</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Example-Guided_LLM_Scoring</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Shower</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>59</v>
-      </c>
-      <c r="G33" t="n">
-        <v>5</v>
-      </c>
-      <c r="H33" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="I33" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="J33" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="K33" t="n">
-        <v>1</v>
-      </c>
-      <c r="L33" t="n">
-        <v>1</v>
-      </c>
-      <c r="M33" t="n">
-        <v>0.8066</v>
-      </c>
-      <c r="N33" t="n">
-        <v>1</v>
-      </c>
-      <c r="O33" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>